<commit_message>
results: refresh execution evidence and metrics
</commit_message>
<xml_diff>
--- a/Report Test subject/test-cases/api/OSMS-API-Test-Cases.xlsx
+++ b/Report Test subject/test-cases/api/OSMS-API-Test-Cases.xlsx
@@ -8,22 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\Online-Sales-Management-System\Report Test subject\test-cases\api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{118F0792-0935-4A24-BBDD-934F817506B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF992C43-D382-412E-A196-6C5176F119A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7B0EA36C-9127-40BF-86EC-90E3FE9E1EE6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5D4903F0-BE73-4DAC-8AAE-21EEC2F57EA8}"/>
   </bookViews>
   <sheets>
-    <sheet name="API Test Cases" sheetId="1" r:id="rId1"/>
+    <sheet name="OSMS-API-Test-Cases" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Test Cases'!$A$1:$P$20</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="151">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -112,10 +109,10 @@
     <t>JSON response contains non-empty fields for status, service, serverTimeUtc, and version; status value is ok.</t>
   </si>
   <si>
-    <t>PENDING REAL EXECUTION</t>
-  </si>
-  <si>
-    <t>Not Run</t>
+    <t>Health endpoint returned 200 OK and all Newman assertions for status, service, serverTimeUtc, and version passed in the full collection rerun.</t>
+  </si>
+  <si>
+    <t>Pass</t>
   </si>
   <si>
     <t>TC-API-CAT-001</t>
@@ -149,6 +146,9 @@
   </si>
   <si>
     <t>JSON response contains page, pageSize, totalItems, totalPages, and items array; items array contains active products with fields such as id, sku, name, categoryName, brandName, salePrice, stockOnHand.</t>
+  </si>
+  <si>
+    <t>Request returned the expected HTTP status and passed all Newman assertions in the full collection run on 2026-04-06.</t>
   </si>
   <si>
     <t>TC-API-CAT-002</t>
@@ -479,7 +479,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="14"/>
       <color theme="1"/>
@@ -615,15 +615,8 @@
       <family val="2"/>
       <charset val="163"/>
     </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
   </fonts>
-  <fills count="34">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -803,14 +796,8 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="22"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -925,21 +912,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -985,17 +957,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1370,1030 +1333,1011 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95BCD6AC-1E22-4300-876E-520619059722}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A47BC6F-E786-427D-AB6F-8EA054BF5FBF}">
   <dimension ref="A1:P20"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="2" width="16.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="38.77734375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.77734375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="12.77734375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="28.77734375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.77734375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="15.77734375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="10.77734375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="28.77734375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="30.77734375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="70.77734375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="16.77734375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="80.77734375" style="1" customWidth="1"/>
-    <col min="15" max="15" width="24.77734375" style="1" customWidth="1"/>
-    <col min="16" max="16" width="12.77734375" style="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.88671875" style="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" t="s">
         <v>24</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" t="s">
         <v>26</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" t="s">
         <v>27</v>
       </c>
-      <c r="M2" s="3">
+      <c r="M2">
         <v>200</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="N2" t="s">
         <v>28</v>
       </c>
-      <c r="O2" s="3" t="s">
+      <c r="O2" t="s">
         <v>29</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="P2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>31</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" t="s">
         <v>33</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" t="s">
         <v>36</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" t="s">
         <v>22</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" t="s">
         <v>37</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" t="s">
         <v>38</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" t="s">
         <v>39</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" t="s">
         <v>40</v>
       </c>
-      <c r="M3" s="3">
+      <c r="M3">
         <v>200</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="N3" t="s">
         <v>41</v>
       </c>
-      <c r="O3" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P3" s="3" t="s">
+      <c r="O3" t="s">
+        <v>42</v>
+      </c>
+      <c r="P3" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K4" t="s">
+        <v>46</v>
+      </c>
+      <c r="L4" t="s">
+        <v>47</v>
+      </c>
+      <c r="M4">
+        <v>200</v>
+      </c>
+      <c r="N4" t="s">
+        <v>48</v>
+      </c>
+      <c r="O4" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="P4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="C5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D5" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E5" t="s">
         <v>35</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F5" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G5" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H5" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I5" t="s">
         <v>37</v>
       </c>
-      <c r="J4" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="M4" s="3">
+      <c r="J5" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" t="s">
+        <v>52</v>
+      </c>
+      <c r="L5" t="s">
+        <v>53</v>
+      </c>
+      <c r="M5">
         <v>200</v>
       </c>
-      <c r="N4" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P4" s="3" t="s">
+      <c r="N5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O5" t="s">
+        <v>42</v>
+      </c>
+      <c r="P5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B5" s="3" t="s">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D5" s="3" t="s">
+      <c r="C6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D6" t="s">
         <v>34</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E6" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F6" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G6" t="s">
         <v>22</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H6" t="s">
         <v>23</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I6" t="s">
         <v>37</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="M5" s="3">
+      <c r="J6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K6" t="s">
+        <v>58</v>
+      </c>
+      <c r="L6" t="s">
+        <v>59</v>
+      </c>
+      <c r="M6">
         <v>200</v>
       </c>
-      <c r="N5" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P5" s="3" t="s">
+      <c r="N6" t="s">
+        <v>60</v>
+      </c>
+      <c r="O6" t="s">
+        <v>42</v>
+      </c>
+      <c r="P6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="3" t="s">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="C7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D7" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E7" t="s">
         <v>35</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F7" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G7" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H7" t="s">
         <v>23</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I7" t="s">
         <v>37</v>
       </c>
-      <c r="J6" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="M6" s="3">
+      <c r="J7" t="s">
+        <v>63</v>
+      </c>
+      <c r="K7" t="s">
+        <v>64</v>
+      </c>
+      <c r="L7" t="s">
+        <v>65</v>
+      </c>
+      <c r="M7">
         <v>200</v>
       </c>
-      <c r="N6" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P6" s="3" t="s">
+      <c r="N7" t="s">
+        <v>66</v>
+      </c>
+      <c r="O7" t="s">
+        <v>42</v>
+      </c>
+      <c r="P7" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="75" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D7" s="3" t="s">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" t="s">
+        <v>68</v>
+      </c>
+      <c r="C8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E8" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8" t="s">
+        <v>37</v>
+      </c>
+      <c r="J8" t="s">
+        <v>71</v>
+      </c>
+      <c r="K8" t="s">
+        <v>72</v>
+      </c>
+      <c r="L8" t="s">
+        <v>73</v>
+      </c>
+      <c r="M8">
+        <v>400</v>
+      </c>
+      <c r="N8" t="s">
+        <v>74</v>
+      </c>
+      <c r="O8" t="s">
+        <v>42</v>
+      </c>
+      <c r="P8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" t="s">
+        <v>37</v>
+      </c>
+      <c r="J9" t="s">
+        <v>77</v>
+      </c>
+      <c r="K9" t="s">
+        <v>78</v>
+      </c>
+      <c r="L9" t="s">
+        <v>79</v>
+      </c>
+      <c r="M9">
+        <v>400</v>
+      </c>
+      <c r="N9" t="s">
+        <v>80</v>
+      </c>
+      <c r="O9" t="s">
+        <v>42</v>
+      </c>
+      <c r="P9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" t="s">
+        <v>82</v>
+      </c>
+      <c r="D10" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10" t="s">
+        <v>23</v>
+      </c>
+      <c r="I10" t="s">
+        <v>37</v>
+      </c>
+      <c r="J10" t="s">
+        <v>83</v>
+      </c>
+      <c r="K10" t="s">
+        <v>84</v>
+      </c>
+      <c r="L10" t="s">
+        <v>85</v>
+      </c>
+      <c r="M10">
+        <v>400</v>
+      </c>
+      <c r="N10" t="s">
+        <v>80</v>
+      </c>
+      <c r="O10" t="s">
+        <v>42</v>
+      </c>
+      <c r="P10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" t="s">
+        <v>36</v>
+      </c>
+      <c r="G11" t="s">
+        <v>22</v>
+      </c>
+      <c r="H11" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" t="s">
+        <v>37</v>
+      </c>
+      <c r="J11" t="s">
+        <v>88</v>
+      </c>
+      <c r="K11" t="s">
+        <v>89</v>
+      </c>
+      <c r="L11" t="s">
+        <v>90</v>
+      </c>
+      <c r="M11">
+        <v>400</v>
+      </c>
+      <c r="N11" t="s">
+        <v>91</v>
+      </c>
+      <c r="O11" t="s">
+        <v>42</v>
+      </c>
+      <c r="P11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" t="s">
+        <v>68</v>
+      </c>
+      <c r="C12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" t="s">
+        <v>36</v>
+      </c>
+      <c r="G12" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" t="s">
+        <v>37</v>
+      </c>
+      <c r="J12" t="s">
+        <v>94</v>
+      </c>
+      <c r="K12" t="s">
+        <v>95</v>
+      </c>
+      <c r="L12" t="s">
+        <v>96</v>
+      </c>
+      <c r="M12">
+        <v>400</v>
+      </c>
+      <c r="N12" t="s">
+        <v>97</v>
+      </c>
+      <c r="O12" t="s">
+        <v>42</v>
+      </c>
+      <c r="P12" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F13" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" t="s">
+        <v>22</v>
+      </c>
+      <c r="H13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" t="s">
+        <v>37</v>
+      </c>
+      <c r="J13" t="s">
+        <v>100</v>
+      </c>
+      <c r="K13" t="s">
+        <v>101</v>
+      </c>
+      <c r="L13" t="s">
+        <v>102</v>
+      </c>
+      <c r="M13">
+        <v>400</v>
+      </c>
+      <c r="N13" t="s">
+        <v>103</v>
+      </c>
+      <c r="O13" t="s">
+        <v>42</v>
+      </c>
+      <c r="P13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>104</v>
+      </c>
+      <c r="B14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" t="s">
+        <v>36</v>
+      </c>
+      <c r="G14" t="s">
+        <v>22</v>
+      </c>
+      <c r="H14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" t="s">
+        <v>37</v>
+      </c>
+      <c r="J14" t="s">
+        <v>106</v>
+      </c>
+      <c r="K14" t="s">
+        <v>107</v>
+      </c>
+      <c r="L14" t="s">
+        <v>108</v>
+      </c>
+      <c r="M14">
+        <v>400</v>
+      </c>
+      <c r="N14" t="s">
+        <v>109</v>
+      </c>
+      <c r="O14" t="s">
+        <v>42</v>
+      </c>
+      <c r="P14" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" t="s">
+        <v>111</v>
+      </c>
+      <c r="D15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" t="s">
+        <v>112</v>
+      </c>
+      <c r="F15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15" t="s">
+        <v>22</v>
+      </c>
+      <c r="H15" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" t="s">
+        <v>37</v>
+      </c>
+      <c r="J15" t="s">
+        <v>113</v>
+      </c>
+      <c r="K15" t="s">
+        <v>114</v>
+      </c>
+      <c r="L15" t="s">
+        <v>115</v>
+      </c>
+      <c r="M15">
+        <v>400</v>
+      </c>
+      <c r="N15" t="s">
+        <v>116</v>
+      </c>
+      <c r="O15" t="s">
+        <v>42</v>
+      </c>
+      <c r="P15" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>117</v>
+      </c>
+      <c r="B16" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" t="s">
+        <v>119</v>
+      </c>
+      <c r="D16" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" t="s">
         <v>35</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G7" s="3" t="s">
+      <c r="F16" t="s">
+        <v>120</v>
+      </c>
+      <c r="G16" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="3" t="s">
+      <c r="H16" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I16" t="s">
         <v>37</v>
       </c>
-      <c r="J7" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="M7" s="3">
+      <c r="J16" t="s">
+        <v>121</v>
+      </c>
+      <c r="K16" t="s">
+        <v>122</v>
+      </c>
+      <c r="L16" t="s">
+        <v>123</v>
+      </c>
+      <c r="M16">
         <v>200</v>
       </c>
-      <c r="N7" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P7" s="3" t="s">
+      <c r="N16" t="s">
+        <v>124</v>
+      </c>
+      <c r="O16" t="s">
+        <v>42</v>
+      </c>
+      <c r="P16" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" s="3" t="s">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>125</v>
+      </c>
+      <c r="B17" t="s">
+        <v>126</v>
+      </c>
+      <c r="C17" t="s">
+        <v>127</v>
+      </c>
+      <c r="D17" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G8" s="3" t="s">
+      <c r="E17" t="s">
+        <v>70</v>
+      </c>
+      <c r="F17" t="s">
+        <v>120</v>
+      </c>
+      <c r="G17" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H17" t="s">
         <v>23</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I17" t="s">
         <v>37</v>
       </c>
-      <c r="J8" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="M8" s="3">
+      <c r="J17" t="s">
+        <v>128</v>
+      </c>
+      <c r="K17" t="s">
+        <v>129</v>
+      </c>
+      <c r="L17" t="s">
+        <v>130</v>
+      </c>
+      <c r="M17">
         <v>400</v>
       </c>
-      <c r="N8" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P8" s="3" t="s">
+      <c r="N17" t="s">
+        <v>131</v>
+      </c>
+      <c r="O17" t="s">
+        <v>42</v>
+      </c>
+      <c r="P17" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D9" s="3" t="s">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>132</v>
+      </c>
+      <c r="B18" t="s">
+        <v>126</v>
+      </c>
+      <c r="C18" t="s">
+        <v>133</v>
+      </c>
+      <c r="D18" t="s">
         <v>34</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G9" s="3" t="s">
+      <c r="E18" t="s">
+        <v>112</v>
+      </c>
+      <c r="F18" t="s">
+        <v>120</v>
+      </c>
+      <c r="G18" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H18" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="I18" t="s">
         <v>37</v>
       </c>
-      <c r="J9" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="M9" s="3">
-        <v>400</v>
-      </c>
-      <c r="N9" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="O9" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P9" s="3" t="s">
+      <c r="J18" t="s">
+        <v>134</v>
+      </c>
+      <c r="K18" t="s">
+        <v>135</v>
+      </c>
+      <c r="L18" t="s">
+        <v>136</v>
+      </c>
+      <c r="M18">
+        <v>404</v>
+      </c>
+      <c r="N18" t="s">
+        <v>137</v>
+      </c>
+      <c r="O18" t="s">
+        <v>42</v>
+      </c>
+      <c r="P18" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" s="3" t="s">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>138</v>
+      </c>
+      <c r="B19" t="s">
+        <v>139</v>
+      </c>
+      <c r="C19" t="s">
+        <v>140</v>
+      </c>
+      <c r="D19" t="s">
         <v>34</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G10" s="3" t="s">
+      <c r="E19" t="s">
+        <v>35</v>
+      </c>
+      <c r="F19" t="s">
+        <v>141</v>
+      </c>
+      <c r="G19" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H19" t="s">
         <v>23</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="I19" t="s">
         <v>37</v>
       </c>
-      <c r="J10" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="M10" s="3">
-        <v>400</v>
-      </c>
-      <c r="N10" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P10" s="3" t="s">
+      <c r="J19" t="s">
+        <v>25</v>
+      </c>
+      <c r="K19" t="s">
+        <v>142</v>
+      </c>
+      <c r="L19" t="s">
+        <v>143</v>
+      </c>
+      <c r="M19">
+        <v>200</v>
+      </c>
+      <c r="N19" t="s">
+        <v>144</v>
+      </c>
+      <c r="O19" t="s">
+        <v>42</v>
+      </c>
+      <c r="P19" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D11" s="3" t="s">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>145</v>
+      </c>
+      <c r="B20" t="s">
+        <v>139</v>
+      </c>
+      <c r="C20" t="s">
+        <v>146</v>
+      </c>
+      <c r="D20" t="s">
         <v>34</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G11" s="3" t="s">
+      <c r="E20" t="s">
+        <v>35</v>
+      </c>
+      <c r="F20" t="s">
+        <v>147</v>
+      </c>
+      <c r="G20" t="s">
         <v>22</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="H20" t="s">
         <v>23</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="I20" t="s">
         <v>37</v>
       </c>
-      <c r="J11" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="M11" s="3">
-        <v>400</v>
-      </c>
-      <c r="N11" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="O11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P11" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="M12" s="3">
-        <v>400</v>
-      </c>
-      <c r="N12" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="M13" s="3">
-        <v>400</v>
-      </c>
-      <c r="N13" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="O13" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P13" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="M14" s="3">
-        <v>400</v>
-      </c>
-      <c r="N14" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="O14" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P14" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="L15" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="M15" s="3">
-        <v>400</v>
-      </c>
-      <c r="N15" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="O15" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P15" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="L16" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="M16" s="3">
+      <c r="J20" t="s">
+        <v>25</v>
+      </c>
+      <c r="K20" t="s">
+        <v>148</v>
+      </c>
+      <c r="L20" t="s">
+        <v>149</v>
+      </c>
+      <c r="M20">
         <v>200</v>
       </c>
-      <c r="N16" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="O16" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P16" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="K17" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="L17" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="M17" s="3">
-        <v>400</v>
-      </c>
-      <c r="N17" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="O17" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P17" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="L18" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="M18" s="3">
-        <v>404</v>
-      </c>
-      <c r="N18" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="O18" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P18" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K19" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="M19" s="3">
-        <v>200</v>
-      </c>
-      <c r="N19" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="O19" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P19" s="3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" ht="56.25" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J20" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K20" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="M20" s="3">
-        <v>200</v>
-      </c>
-      <c r="N20" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="O20" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P20" s="3" t="s">
+      <c r="N20" t="s">
+        <v>150</v>
+      </c>
+      <c r="O20" t="s">
+        <v>42</v>
+      </c>
+      <c r="P20" t="s">
         <v>30</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P20" xr:uid="{95BCD6AC-1E22-4300-876E-520619059722}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>